<commit_message>
adjusted codes and test run
</commit_message>
<xml_diff>
--- a/Maps/sdtm_mapping_paths.xlsx
+++ b/Maps/sdtm_mapping_paths.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\USDM_SDTM_mapper\Maps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5FEC9C-A9F8-49F6-BC6C-2225D8EE8F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FC400D-129C-44D1-A2A8-888DC3F7B971}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8790" yWindow="-18810" windowWidth="38700" windowHeight="15225" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="740" windowWidth="19180" windowHeight="11260" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="1" r:id="rId1"/>
@@ -1290,24 +1290,6 @@
     <t>study.versions.studyDesigns[studyType.code="C16084"].samplingMethod.decode</t>
   </si>
   <si>
-    <t>study.versions.studyDesigns.objectives[level.code="C85826"].{id: text}</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.objectives[level.code="C85827"].{id: text}</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.objectives[level.code="C163559"].{id: text}</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.objectives[level.code="C85826"].{id: objectives.endpoint.text}</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.objectives[level.code="C85827"].{id: objectives.endpoint.text}</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.objectives[level.code="C163559"].{id: objectives.endpoint.text}</t>
-  </si>
-  <si>
     <t>Fixed content</t>
   </si>
   <si>
@@ -1320,39 +1302,6 @@
     <t>Minimum Response Duration</t>
   </si>
   <si>
-    <t>study.versions.studyInterventions.{id: minimumResponseDuration.value &amp; " " &amp; minimumResponseDuration.unit.standardCode.decode}</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions[role.code="C165822"].{id: label}</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions[role.code="C41161"].{id: label}</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions{id: type.decode}</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions{id: administrations.duration.quantity.value &amp; " " &amp; administrations.duration.quantity.unit.standardCode.decode}</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions{id: role[code="C753"].decode ? role[code="C753"].decode : role[code="C68609"].decode}</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions{id: administrations.administrableProduct.administrableDoseForm.standardCode.decode}</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions{id: administrations.dose.value}</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions{id: administrations.dose.unit.standardCode.decode}</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions{id: administrations.frequency.standardCode.decode}</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions[role.code="C68609"].{id: label}</t>
-  </si>
-  <si>
     <t>TS</t>
   </si>
   <si>
@@ -1471,9 +1420,6 @@
   </si>
   <si>
     <t>study.study.versions.studyDesigns.studyPhase.standardCode.codeSystemVersion</t>
-  </si>
-  <si>
-    <t>study.versions.studyInterventions{id: administrations.route.standardCode.decode}</t>
   </si>
   <si>
     <t>study.versions.studyInterventions{id: administrations.route.standardCode.code}</t>
@@ -1597,9 +1543,6 @@
   </si>
   <si>
     <t>study.versions.studyDesigns[studyType.code="C98388"].subTypes.{id: codeSystemVersion}</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.indications.{id: label}</t>
   </si>
   <si>
     <t>The name of the original mapping in DDF USDM v4.0</t>
@@ -1974,6 +1917,63 @@
       </rPr>
       <t xml:space="preserve"> ? "Y" : ""</t>
     </r>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions[role.code="C68609"].{name: label}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions.{name: minimumResponseDuration.value &amp; " " &amp; minimumResponseDuration.unit.standardCode.decode}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions[role.code="C165822"].{name: label}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions{name: administrations.dose.value}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions{name: administrations.administrableProduct.administrableDoseForm.standardCode.decode}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions{name: administrations.frequency.standardCode.decode}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions{name: administrations.dose.unit.standardCode.decode}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions{name: type.decode}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions{name: administrations.duration.quantity.value &amp; " " &amp; administrations.duration.quantity.unit.standardCode.decode}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions{name: administrations.route.standardCode.decode}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions{name: role[code="C753"].decode ? role[code="C753"].decode : role[code="C68609"].decode}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions[role.code="C41161"].{name: label}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives[level.code="C163559"].{name: text}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives[level.code="C85826"].{name: text}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives[level.code="C85827"].{name: text}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives[level.code="C163559"].{name: objectives.endpoint.text}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives[level.code="C85826"].{name: objectives.endpoint.text}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives[level.code="C85827"].{name: objectives.endpoint.text}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.indications.{id: label}</t>
   </si>
 </sst>
 </file>
@@ -2524,7 +2524,7 @@
         <v>40</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>471</v>
+        <v>452</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="31" x14ac:dyDescent="0.35">
@@ -2532,23 +2532,23 @@
         <v>355</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>473</v>
+        <v>454</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="31" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>472</v>
+        <v>453</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>474</v>
+        <v>455</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="31" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>475</v>
+        <v>456</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>476</v>
+        <v>457</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -2578,15 +2578,15 @@
         <v>348</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>477</v>
+        <v>458</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>478</v>
+        <v>459</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>479</v>
+        <v>460</v>
       </c>
     </row>
   </sheetData>
@@ -2634,7 +2634,7 @@
         <v>355</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -2657,7 +2657,7 @@
         <v>38</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>496</v>
+        <v>477</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -2683,7 +2683,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>459</v>
+        <v>441</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -2709,7 +2709,7 @@
         <v>316</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>460</v>
+        <v>442</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -2732,7 +2732,7 @@
         <v>317</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>461</v>
+        <v>443</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2755,7 +2755,7 @@
         <v>318</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>493</v>
+        <v>474</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="118" customHeight="1" x14ac:dyDescent="0.35">
@@ -2778,7 +2778,7 @@
         <v>319</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>492</v>
+        <v>473</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -2801,7 +2801,7 @@
         <v>320</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>494</v>
+        <v>475</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
@@ -2864,7 +2864,7 @@
         <v>322</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>495</v>
+        <v>476</v>
       </c>
     </row>
   </sheetData>
@@ -2910,7 +2910,7 @@
         <v>355</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="58" x14ac:dyDescent="0.35">
@@ -2933,7 +2933,7 @@
         <v>38</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>496</v>
+        <v>477</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="1"/>
@@ -2959,7 +2959,7 @@
       <c r="F3" s="10"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>480</v>
+        <v>461</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -2985,7 +2985,7 @@
         <v>342</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>481</v>
+        <v>462</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3008,7 +3008,7 @@
         <v>343</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>482</v>
+        <v>463</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3031,7 +3031,7 @@
         <v>323</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>483</v>
+        <v>464</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3054,7 +3054,7 @@
         <v>324</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>484</v>
+        <v>465</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3120,7 +3120,7 @@
         <v>355</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -3143,7 +3143,7 @@
         <v>38</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>496</v>
+        <v>477</v>
       </c>
       <c r="H2" s="8"/>
     </row>
@@ -3166,7 +3166,7 @@
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
       <c r="H3" s="8" t="s">
-        <v>486</v>
+        <v>467</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -3189,7 +3189,7 @@
         <v>61</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>491</v>
+        <v>472</v>
       </c>
       <c r="H4" s="8"/>
     </row>
@@ -3213,7 +3213,7 @@
         <v>64</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="H5" s="8"/>
     </row>
@@ -3237,7 +3237,7 @@
         <v>66</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>488</v>
+        <v>469</v>
       </c>
       <c r="H6" s="8"/>
     </row>
@@ -3261,7 +3261,7 @@
         <v>316</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>460</v>
+        <v>442</v>
       </c>
       <c r="H7" s="8"/>
     </row>
@@ -3285,7 +3285,7 @@
         <v>317</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>461</v>
+        <v>443</v>
       </c>
       <c r="H8" s="8"/>
     </row>
@@ -3309,7 +3309,7 @@
         <v>72</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>489</v>
+        <v>470</v>
       </c>
       <c r="H9" s="8"/>
     </row>
@@ -3333,7 +3333,7 @@
         <v>74</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>490</v>
+        <v>471</v>
       </c>
       <c r="H10" s="8"/>
     </row>
@@ -3390,7 +3390,7 @@
         <v>355</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="I1" s="15"/>
       <c r="J1" s="15"/>
@@ -3421,7 +3421,7 @@
         <v>38</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>496</v>
+        <v>477</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3443,7 +3443,7 @@
       <c r="F3" s="14"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>451</v>
+        <v>433</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3466,7 +3466,7 @@
         <v>78</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>452</v>
+        <v>434</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -3489,7 +3489,7 @@
         <v>80</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>457</v>
+        <v>439</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3512,7 +3512,7 @@
         <v>82</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>453</v>
+        <v>435</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3535,7 +3535,7 @@
         <v>84</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>454</v>
+        <v>436</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3577,7 +3577,7 @@
         <v>88</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>458</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>
@@ -3624,7 +3624,7 @@
         <v>355</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="J1" s="15"/>
       <c r="K1" s="15"/>
@@ -3654,7 +3654,7 @@
         <v>38</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>496</v>
+        <v>477</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
@@ -3676,7 +3676,7 @@
       <c r="F3" s="10"/>
       <c r="G3" s="10"/>
       <c r="H3" s="9" t="s">
-        <v>389</v>
+        <v>372</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
@@ -3832,7 +3832,7 @@
         <v>106</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -3855,7 +3855,7 @@
         <v>344</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
     </row>
   </sheetData>
@@ -3901,19 +3901,19 @@
         <v>40</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>390</v>
+        <v>373</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>391</v>
+        <v>374</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>392</v>
+        <v>375</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>393</v>
+        <v>376</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>394</v>
+        <v>377</v>
       </c>
       <c r="L1" s="15"/>
       <c r="M1" s="15"/>
@@ -3956,7 +3956,7 @@
         <v>327</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>455</v>
+        <v>437</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="87" x14ac:dyDescent="0.35">
@@ -3975,10 +3975,10 @@
         <v>328</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>456</v>
+        <v>438</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>436</v>
+        <v>418</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="58" x14ac:dyDescent="0.35">
@@ -4045,7 +4045,7 @@
       </c>
       <c r="F7" s="17"/>
       <c r="G7" s="5" t="s">
-        <v>388</v>
+        <v>482</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4088,7 +4088,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
         <v>139</v>
       </c>
@@ -4105,10 +4105,10 @@
         <v>142</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>378</v>
+        <v>483</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4131,10 +4131,10 @@
         <v>331</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="16" t="s">
         <v>147</v>
       </c>
@@ -4150,7 +4150,7 @@
         <v>147</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4173,7 +4173,7 @@
         <v>332</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>385</v>
+        <v>485</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4196,7 +4196,7 @@
         <v>153</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>384</v>
+        <v>486</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="58" x14ac:dyDescent="0.35">
@@ -4219,16 +4219,16 @@
         <v>333</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>387</v>
+        <v>487</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>397</v>
+        <v>380</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>398</v>
+        <v>381</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>399</v>
+        <v>382</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="58" x14ac:dyDescent="0.35">
@@ -4251,19 +4251,19 @@
         <v>334</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>386</v>
+        <v>488</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>400</v>
+        <v>383</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>401</v>
+        <v>384</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="16" t="s">
         <v>162</v>
       </c>
@@ -4279,10 +4279,10 @@
         <v>162</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="16" t="s">
         <v>165</v>
       </c>
@@ -4313,13 +4313,13 @@
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="17" t="s">
-        <v>438</v>
+        <v>420</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="101.5" x14ac:dyDescent="0.35">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A20" s="16" t="s">
         <v>171</v>
       </c>
@@ -4335,7 +4335,7 @@
         <v>335</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>470</v>
+        <v>500</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4357,13 +4357,13 @@
         <v>361</v>
       </c>
       <c r="I21" s="20" t="s">
-        <v>403</v>
+        <v>386</v>
       </c>
       <c r="J21" s="20" t="s">
-        <v>404</v>
+        <v>387</v>
       </c>
       <c r="K21" s="20" t="s">
-        <v>405</v>
+        <v>388</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4386,16 +4386,16 @@
         <v>177</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>381</v>
+        <v>489</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>406</v>
+        <v>389</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>407</v>
+        <v>390</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>408</v>
+        <v>391</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="58" x14ac:dyDescent="0.35">
@@ -4414,10 +4414,10 @@
         <v>352</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>409</v>
+        <v>392</v>
       </c>
       <c r="H23" t="s">
-        <v>395</v>
+        <v>378</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4436,10 +4436,10 @@
         <v>336</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="16" t="s">
         <v>186</v>
       </c>
@@ -4455,7 +4455,7 @@
         <v>189</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>485</v>
+        <v>466</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4474,7 +4474,7 @@
         <v>190</v>
       </c>
       <c r="G26" s="20" t="s">
-        <v>410</v>
+        <v>393</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4513,10 +4513,10 @@
         <v>199</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="16" t="s">
         <v>202</v>
       </c>
@@ -4536,10 +4536,10 @@
         <v>205</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="16" t="s">
         <v>206</v>
       </c>
@@ -4559,7 +4559,7 @@
         <v>209</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>369</v>
+        <v>496</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4581,13 +4581,13 @@
         <v>364</v>
       </c>
       <c r="I31" t="s">
-        <v>411</v>
+        <v>394</v>
       </c>
       <c r="J31" t="s">
-        <v>412</v>
+        <v>395</v>
       </c>
       <c r="K31" t="s">
-        <v>413</v>
+        <v>396</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4609,16 +4609,16 @@
         <v>365</v>
       </c>
       <c r="I32" s="20" t="s">
-        <v>414</v>
+        <v>397</v>
       </c>
       <c r="J32" s="20" t="s">
-        <v>415</v>
+        <v>398</v>
       </c>
       <c r="K32" s="20" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A33" s="16" t="s">
         <v>216</v>
       </c>
@@ -4656,16 +4656,16 @@
         <v>367</v>
       </c>
       <c r="I34" s="20" t="s">
-        <v>417</v>
+        <v>400</v>
       </c>
       <c r="J34" s="20" t="s">
-        <v>418</v>
+        <v>401</v>
       </c>
       <c r="K34" s="20" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A35" s="16" t="s">
         <v>222</v>
       </c>
@@ -4685,10 +4685,10 @@
         <v>222</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="16" t="s">
         <v>227</v>
       </c>
@@ -4708,10 +4708,10 @@
         <v>227</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="16" t="s">
         <v>230</v>
       </c>
@@ -4731,7 +4731,7 @@
         <v>230</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>372</v>
+        <v>499</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4752,10 +4752,10 @@
         <v>233</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="16" t="s">
         <v>236</v>
       </c>
@@ -4771,10 +4771,10 @@
         <v>236</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="116" x14ac:dyDescent="0.35">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A40" s="16" t="s">
         <v>239</v>
       </c>
@@ -4793,7 +4793,7 @@
         <v>363</v>
       </c>
       <c r="H40" t="s">
-        <v>395</v>
+        <v>378</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4814,10 +4814,10 @@
         <v>339</v>
       </c>
       <c r="G41" s="20" t="s">
-        <v>382</v>
+        <v>490</v>
       </c>
       <c r="H41" t="s">
-        <v>395</v>
+        <v>378</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4836,10 +4836,10 @@
         <v>248</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="16" t="s">
         <v>249</v>
       </c>
@@ -4855,7 +4855,7 @@
         <v>252</v>
       </c>
       <c r="G43" s="20" t="s">
-        <v>442</v>
+        <v>424</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4898,16 +4898,16 @@
         <v>258</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>429</v>
+        <v>491</v>
       </c>
       <c r="I45" s="5" t="s">
-        <v>430</v>
+        <v>412</v>
       </c>
       <c r="J45" s="5" t="s">
-        <v>431</v>
+        <v>413</v>
       </c>
       <c r="K45" s="5" t="s">
-        <v>432</v>
+        <v>414</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="58" x14ac:dyDescent="0.35">
@@ -4930,10 +4930,10 @@
         <v>261</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="16" t="s">
         <v>265</v>
       </c>
@@ -4949,10 +4949,10 @@
         <v>265</v>
       </c>
       <c r="G47" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" s="16" t="s">
         <v>268</v>
       </c>
@@ -4968,7 +4968,7 @@
         <v>340</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>434</v>
+        <v>416</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5005,10 +5005,10 @@
         <v>341</v>
       </c>
       <c r="G50" s="18" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="16" t="s">
         <v>277</v>
       </c>
@@ -5024,19 +5024,19 @@
         <v>280</v>
       </c>
       <c r="G51" t="s">
-        <v>443</v>
+        <v>425</v>
       </c>
       <c r="I51" t="s">
-        <v>444</v>
+        <v>426</v>
       </c>
       <c r="J51" t="s">
-        <v>445</v>
+        <v>427</v>
       </c>
       <c r="K51" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" ht="145" x14ac:dyDescent="0.35">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A52" s="16" t="s">
         <v>281</v>
       </c>
@@ -5055,13 +5055,13 @@
         <v>362</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>420</v>
+        <v>403</v>
       </c>
       <c r="J52" s="5" t="s">
-        <v>421</v>
+        <v>404</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>422</v>
+        <v>405</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
@@ -5080,16 +5080,16 @@
         <v>288</v>
       </c>
       <c r="G53" s="20" t="s">
-        <v>383</v>
+        <v>492</v>
       </c>
       <c r="I53" s="20" t="s">
-        <v>423</v>
+        <v>406</v>
       </c>
       <c r="J53" s="20" t="s">
-        <v>424</v>
+        <v>407</v>
       </c>
       <c r="K53" s="20" t="s">
-        <v>425</v>
+        <v>408</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5108,16 +5108,16 @@
         <v>289</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>447</v>
+        <v>429</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>448</v>
+        <v>430</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>449</v>
+        <v>431</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>450</v>
+        <v>432</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -5138,19 +5138,19 @@
         <v>295</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>462</v>
+        <v>444</v>
       </c>
       <c r="I55" s="5" t="s">
-        <v>464</v>
+        <v>446</v>
       </c>
       <c r="J55" s="5" t="s">
-        <v>465</v>
+        <v>447</v>
       </c>
       <c r="K55" s="5" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="16" t="s">
         <v>297</v>
       </c>
@@ -5169,7 +5169,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="16" t="s">
         <v>301</v>
       </c>
@@ -5188,16 +5188,16 @@
         <v>360</v>
       </c>
       <c r="H57" s="16" t="s">
-        <v>395</v>
+        <v>378</v>
       </c>
       <c r="I57" t="s">
-        <v>426</v>
+        <v>409</v>
       </c>
       <c r="J57" t="s">
-        <v>427</v>
+        <v>410</v>
       </c>
       <c r="K57" t="s">
-        <v>428</v>
+        <v>411</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -5220,10 +5220,10 @@
         <v>308</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>380</v>
+        <v>493</v>
       </c>
       <c r="H58" s="16" t="s">
-        <v>396</v>
+        <v>379</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -5242,16 +5242,16 @@
         <v>312</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>463</v>
+        <v>445</v>
       </c>
       <c r="I59" s="5" t="s">
-        <v>467</v>
+        <v>449</v>
       </c>
       <c r="J59" s="5" t="s">
-        <v>468</v>
+        <v>450</v>
       </c>
       <c r="K59" s="5" t="s">
-        <v>469</v>
+        <v>451</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added ISO 8601 formatting
</commit_message>
<xml_diff>
--- a/Maps/sdtm_mapping_paths.xlsx
+++ b/Maps/sdtm_mapping_paths.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\USDM_SDTM_mapper\Maps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FC400D-129C-44D1-A2A8-888DC3F7B971}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2B1A5AB-4108-433D-952A-2A12AA207CB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="740" windowWidth="19180" windowHeight="11260" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="1" r:id="rId1"/>
@@ -1362,9 +1362,6 @@
     <t>study.versions.studyInterventions{id: type.codeSystemVersion}</t>
   </si>
   <si>
-    <t>study.versions.studyDesigns.scheduleTimelines[mainTimeline=true].plannedDuration.quantity.value &amp; " " &amp; study.versions.studyDesigns.scheduleTimelines[mainTimeline=true].plannedDuration.quantity.unit.standardCode.decode</t>
-  </si>
-  <si>
     <t>$exists(study.versions.studyDesigns.population.cohorts) ? $count(study.versions.studyDesigns.population.cohorts) : ""</t>
   </si>
   <si>
@@ -1495,15 +1492,6 @@
   </si>
   <si>
     <t>study.versions.studyDesigns.eligibilityCriteria{id: notes.codes.decode}</t>
-  </si>
-  <si>
-    <t>$min([study.versions.studyDesigns.population.plannedAge.minValue.value,study.versions.studyDesigns.population.cohorts.plannedAge.minValue.value]) &amp; " " &amp; 
-$distinct(study.versions.studyDesigns.population.plannedAge.minValue.unit.standardCode.decode)
- &amp; " " &amp; $distinct(study.versions.studyDesigns.population.cohorts.plannedAge.minValue.unit.standardCode.decode)</t>
-  </si>
-  <si>
-    <t>$max([study.versions.studyDesigns.population.plannedAge.maxValue.value,study.versions.studyDesigns.population.cohorts.plannedAge.maxValue.value]) &amp; " " &amp; 
-$distinct(study.versions.studyDesigns.population.plannedAge.maxValue.unit.standardCode.decode) &amp; " " &amp; $distinct(study.versions.studyDesigns.population.cohorts.plannedAge.maxValue.unit.standardCode.decode)</t>
   </si>
   <si>
     <t>study.versions.($EligTxt := function($id) {(eligibilityCriterionItems[id=$id].text)}; studyDesigns.eligibilityCriteria{id: $EligTxt(criterionItemId)})</t>
@@ -1922,9 +1910,6 @@
     <t>study.versions.studyInterventions[role.code="C68609"].{name: label}</t>
   </si>
   <si>
-    <t>study.versions.studyInterventions.{name: minimumResponseDuration.value &amp; " " &amp; minimumResponseDuration.unit.standardCode.decode}</t>
-  </si>
-  <si>
     <t>study.versions.studyInterventions[role.code="C165822"].{name: label}</t>
   </si>
   <si>
@@ -1943,9 +1928,6 @@
     <t>study.versions.studyInterventions{name: type.decode}</t>
   </si>
   <si>
-    <t>study.versions.studyInterventions{name: administrations.duration.quantity.value &amp; " " &amp; administrations.duration.quantity.unit.standardCode.decode}</t>
-  </si>
-  <si>
     <t>study.versions.studyInterventions{name: administrations.route.standardCode.decode}</t>
   </si>
   <si>
@@ -1974,6 +1956,24 @@
   </si>
   <si>
     <t>study.versions.studyDesigns.indications.{id: label}</t>
+  </si>
+  <si>
+    <t>"P" &amp; $min([study.versions.studyDesigns.population.plannedAge.minValue.value,study.versions.studyDesigns.population.cohorts.plannedAge.minValue.value]) &amp;  
+$substring($distinct(study.versions.studyDesigns.population.plannedAge.minValue.unit.standardCode.decode),0,1)
+&amp; $substring($distinct(study.versions.studyDesigns.population.cohorts.plannedAge.minValue.unit.standardCode.decode),0,1)</t>
+  </si>
+  <si>
+    <t>"P" &amp; $max([study.versions.studyDesigns.population.plannedAge.maxValue.value,study.versions.studyDesigns.population.cohorts.plannedAge.maxValue.value]) &amp; 
+$substring($distinct(study.versions.studyDesigns.population.plannedAge.maxValue.unit.standardCode.decode),0,1) &amp;  $substring($distinct(study.versions.studyDesigns.population.cohorts.plannedAge.maxValue.unit.standardCode.decode),0,1)</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions.{name: "P" &amp; minimumResponseDuration.value &amp; $substring(minimumResponseDuration.unit.standardCode.decode,1,1)}</t>
+  </si>
+  <si>
+    <t>$exists(study.versions.studyDesigns.scheduleTimelines[mainTimeline=true].plannedDuration.quantity) ? "P" &amp; study.versions.studyDesigns.scheduleTimelines[mainTimeline=true].plannedDuration.quantity.value &amp; $substring(study.versions.studyDesigns.scheduleTimelines[mainTimeline=true].plannedDuration.quantity.unit.standardCode.decode,1,1)</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions{name: administrations.duration.quantity.("P"&amp; value &amp; $substring(unit.standardCode.decode,0,1))}</t>
   </si>
 </sst>
 </file>
@@ -2524,7 +2524,7 @@
         <v>40</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="31" x14ac:dyDescent="0.35">
@@ -2532,23 +2532,23 @@
         <v>355</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="31" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="31" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -2578,15 +2578,15 @@
         <v>348</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
     </row>
   </sheetData>
@@ -2657,7 +2657,7 @@
         <v>38</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -2683,7 +2683,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -2709,7 +2709,7 @@
         <v>316</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -2732,7 +2732,7 @@
         <v>317</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2755,7 +2755,7 @@
         <v>318</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="118" customHeight="1" x14ac:dyDescent="0.35">
@@ -2778,7 +2778,7 @@
         <v>319</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -2801,7 +2801,7 @@
         <v>320</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
@@ -2864,7 +2864,7 @@
         <v>322</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
     </row>
   </sheetData>
@@ -2933,7 +2933,7 @@
         <v>38</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="1"/>
@@ -2959,7 +2959,7 @@
       <c r="F3" s="10"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -2985,7 +2985,7 @@
         <v>342</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3008,7 +3008,7 @@
         <v>343</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3031,7 +3031,7 @@
         <v>323</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3054,7 +3054,7 @@
         <v>324</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3143,7 +3143,7 @@
         <v>38</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="H2" s="8"/>
     </row>
@@ -3166,7 +3166,7 @@
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
       <c r="H3" s="8" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -3189,7 +3189,7 @@
         <v>61</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="H4" s="8"/>
     </row>
@@ -3213,7 +3213,7 @@
         <v>64</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="H5" s="8"/>
     </row>
@@ -3237,7 +3237,7 @@
         <v>66</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="H6" s="8"/>
     </row>
@@ -3261,7 +3261,7 @@
         <v>316</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="H7" s="8"/>
     </row>
@@ -3285,7 +3285,7 @@
         <v>317</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="H8" s="8"/>
     </row>
@@ -3309,7 +3309,7 @@
         <v>72</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="H9" s="8"/>
     </row>
@@ -3333,7 +3333,7 @@
         <v>74</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="H10" s="8"/>
     </row>
@@ -3421,7 +3421,7 @@
         <v>38</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3443,7 +3443,7 @@
       <c r="F3" s="14"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3466,7 +3466,7 @@
         <v>78</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -3489,7 +3489,7 @@
         <v>80</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3512,7 +3512,7 @@
         <v>82</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3535,7 +3535,7 @@
         <v>84</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3577,7 +3577,7 @@
         <v>88</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
   </sheetData>
@@ -3654,7 +3654,7 @@
         <v>38</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
@@ -3956,10 +3956,10 @@
         <v>327</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="87" x14ac:dyDescent="0.35">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A4" s="16" t="s">
         <v>113</v>
       </c>
@@ -3975,10 +3975,10 @@
         <v>328</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>438</v>
+        <v>497</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="58" x14ac:dyDescent="0.35">
@@ -4045,7 +4045,7 @@
       </c>
       <c r="F7" s="17"/>
       <c r="G7" s="5" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4108,7 +4108,7 @@
         <v>371</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>483</v>
+        <v>498</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4131,7 +4131,7 @@
         <v>331</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4150,7 +4150,7 @@
         <v>147</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4173,7 +4173,7 @@
         <v>332</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4196,7 +4196,7 @@
         <v>153</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="58" x14ac:dyDescent="0.35">
@@ -4219,7 +4219,7 @@
         <v>333</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>380</v>
@@ -4251,7 +4251,7 @@
         <v>334</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>383</v>
@@ -4279,7 +4279,7 @@
         <v>162</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4313,10 +4313,10 @@
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="17" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="58" x14ac:dyDescent="0.35">
@@ -4335,7 +4335,7 @@
         <v>335</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4386,7 +4386,7 @@
         <v>177</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>389</v>
@@ -4398,7 +4398,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" ht="87" x14ac:dyDescent="0.35">
       <c r="A23" s="16" t="s">
         <v>180</v>
       </c>
@@ -4414,7 +4414,7 @@
         <v>352</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>392</v>
+        <v>499</v>
       </c>
       <c r="H23" t="s">
         <v>378</v>
@@ -4436,7 +4436,7 @@
         <v>336</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
@@ -4455,7 +4455,7 @@
         <v>189</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4474,7 +4474,7 @@
         <v>190</v>
       </c>
       <c r="G26" s="20" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4513,7 +4513,7 @@
         <v>199</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4536,7 +4536,7 @@
         <v>205</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4559,7 +4559,7 @@
         <v>209</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>496</v>
+        <v>491</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4581,13 +4581,13 @@
         <v>364</v>
       </c>
       <c r="I31" t="s">
+        <v>393</v>
+      </c>
+      <c r="J31" t="s">
         <v>394</v>
       </c>
-      <c r="J31" t="s">
+      <c r="K31" t="s">
         <v>395</v>
-      </c>
-      <c r="K31" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4609,13 +4609,13 @@
         <v>365</v>
       </c>
       <c r="I32" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="J32" s="20" t="s">
         <v>397</v>
       </c>
-      <c r="J32" s="20" t="s">
+      <c r="K32" s="20" t="s">
         <v>398</v>
-      </c>
-      <c r="K32" s="20" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4656,13 +4656,13 @@
         <v>367</v>
       </c>
       <c r="I34" s="20" t="s">
+        <v>399</v>
+      </c>
+      <c r="J34" s="20" t="s">
         <v>400</v>
       </c>
-      <c r="J34" s="20" t="s">
+      <c r="K34" s="20" t="s">
         <v>401</v>
-      </c>
-      <c r="K34" s="20" t="s">
-        <v>402</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4685,7 +4685,7 @@
         <v>222</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4708,7 +4708,7 @@
         <v>227</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4731,7 +4731,7 @@
         <v>230</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>499</v>
+        <v>494</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4752,7 +4752,7 @@
         <v>233</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4771,7 +4771,7 @@
         <v>236</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4814,7 +4814,7 @@
         <v>339</v>
       </c>
       <c r="G41" s="20" t="s">
-        <v>490</v>
+        <v>500</v>
       </c>
       <c r="H41" t="s">
         <v>378</v>
@@ -4836,7 +4836,7 @@
         <v>248</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
@@ -4855,7 +4855,7 @@
         <v>252</v>
       </c>
       <c r="G43" s="20" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4898,16 +4898,16 @@
         <v>258</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="I45" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="J45" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="J45" s="5" t="s">
+      <c r="K45" s="5" t="s">
         <v>413</v>
-      </c>
-      <c r="K45" s="5" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="58" x14ac:dyDescent="0.35">
@@ -4930,7 +4930,7 @@
         <v>261</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
@@ -4949,7 +4949,7 @@
         <v>265</v>
       </c>
       <c r="G47" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4968,7 +4968,7 @@
         <v>340</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5005,7 +5005,7 @@
         <v>341</v>
       </c>
       <c r="G50" s="18" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5024,16 +5024,16 @@
         <v>280</v>
       </c>
       <c r="G51" t="s">
+        <v>424</v>
+      </c>
+      <c r="I51" t="s">
         <v>425</v>
       </c>
-      <c r="I51" t="s">
+      <c r="J51" t="s">
         <v>426</v>
       </c>
-      <c r="J51" t="s">
+      <c r="K51" t="s">
         <v>427</v>
-      </c>
-      <c r="K51" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
@@ -5055,13 +5055,13 @@
         <v>362</v>
       </c>
       <c r="I52" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="J52" s="5" t="s">
         <v>403</v>
       </c>
-      <c r="J52" s="5" t="s">
+      <c r="K52" s="5" t="s">
         <v>404</v>
-      </c>
-      <c r="K52" s="5" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
@@ -5080,16 +5080,16 @@
         <v>288</v>
       </c>
       <c r="G53" s="20" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="I53" s="20" t="s">
+        <v>405</v>
+      </c>
+      <c r="J53" s="20" t="s">
         <v>406</v>
       </c>
-      <c r="J53" s="20" t="s">
+      <c r="K53" s="20" t="s">
         <v>407</v>
-      </c>
-      <c r="K53" s="20" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5108,16 +5108,16 @@
         <v>289</v>
       </c>
       <c r="G54" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="I54" s="5" t="s">
         <v>429</v>
       </c>
-      <c r="I54" s="5" t="s">
+      <c r="J54" s="5" t="s">
         <v>430</v>
       </c>
-      <c r="J54" s="5" t="s">
+      <c r="K54" s="5" t="s">
         <v>431</v>
-      </c>
-      <c r="K54" s="5" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -5138,16 +5138,16 @@
         <v>295</v>
       </c>
       <c r="G55" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="I55" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="J55" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="I55" s="5" t="s">
-        <v>446</v>
-      </c>
-      <c r="J55" s="5" t="s">
-        <v>447</v>
-      </c>
       <c r="K55" s="5" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5191,13 +5191,13 @@
         <v>378</v>
       </c>
       <c r="I57" t="s">
+        <v>408</v>
+      </c>
+      <c r="J57" t="s">
         <v>409</v>
       </c>
-      <c r="J57" t="s">
+      <c r="K57" t="s">
         <v>410</v>
-      </c>
-      <c r="K57" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -5220,7 +5220,7 @@
         <v>308</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
       <c r="H58" s="16" t="s">
         <v>379</v>
@@ -5242,16 +5242,16 @@
         <v>312</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="I59" s="5" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="J59" s="5" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="K59" s="5" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added TA.TABRANCH and TA.TATRANS
</commit_message>
<xml_diff>
--- a/Maps/sdtm_mapping_paths.xlsx
+++ b/Maps/sdtm_mapping_paths.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\USDM_SDTM_mapper\Maps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E02EF51-7ADA-420D-8756-24146F30C2D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01FF7E84-0502-47C2-8DC0-A24DBAEDA929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="500">
   <si>
     <t>Identifier</t>
   </si>
@@ -1884,24 +1884,15 @@
     <t>study.versions.studyInterventions{name: administrations.duration.quantity.("P"&amp; value &amp; $substring(unit.standardCode.decode,0,1))}</t>
   </si>
   <si>
-    <t>Domain</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
-    <t>SasDatasetName</t>
-  </si>
-  <si>
     <t>Repeating</t>
   </si>
   <si>
     <t>IsReferenceData</t>
   </si>
   <si>
-    <t>OID</t>
-  </si>
-  <si>
     <t>Purpose</t>
   </si>
   <si>
@@ -1911,15 +1902,6 @@
     <t>Structure</t>
   </si>
   <si>
-    <t>ArchiveLocationID</t>
-  </si>
-  <si>
-    <t>StandardOID</t>
-  </si>
-  <si>
-    <t>IG.TS</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -1929,48 +1911,18 @@
     <t>One record per trial summary parameter value</t>
   </si>
   <si>
-    <t>LF.TS</t>
-  </si>
-  <si>
-    <t>STD.1</t>
-  </si>
-  <si>
-    <t>IG.TA</t>
-  </si>
-  <si>
-    <t>LF.TA</t>
-  </si>
-  <si>
-    <t>IG.TE</t>
-  </si>
-  <si>
     <t>One record per arm and epoch</t>
   </si>
   <si>
     <t>One record per element</t>
   </si>
   <si>
-    <t>LF.TE</t>
-  </si>
-  <si>
-    <t>IG.TV</t>
-  </si>
-  <si>
     <t>One record per planned visit</t>
   </si>
   <si>
-    <t>LF.TV</t>
-  </si>
-  <si>
-    <t>IG.TI</t>
-  </si>
-  <si>
     <t>One record per eligibility criterion per study version</t>
   </si>
   <si>
-    <t>LF.TI</t>
-  </si>
-  <si>
     <t>TAETORD</t>
   </si>
   <si>
@@ -2011,6 +1963,16 @@
   </si>
   <si>
     <t>Trial Inclusion and Exclusion Criteria</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.characteristics[code in ["C46079","C25689","C147145"]].decode</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.scheduleTimelines.($GetEpochId := function($id) {(instances[id=$id].epochId)}; instances[instanceType="ScheduledDecisionInstance"].
+{epochId: conditionAssignments.condition,"targetEpoch":$GetEpochId(conditionAssignments.conditionTargetId)})</t>
   </si>
 </sst>
 </file>
@@ -2642,226 +2604,137 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC97F1FB-6C60-4A00-8A25-0792299D1D70}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="41" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.90625" customWidth="1"/>
+    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="41" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="22" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="22" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>471</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="D1" s="22" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>497</v>
+      </c>
+      <c r="F1" s="22" t="s">
+        <v>475</v>
+      </c>
+      <c r="G1" s="22" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>341</v>
+      </c>
+      <c r="B2" t="s">
         <v>476</v>
       </c>
-      <c r="E1" s="22" t="s">
-        <v>472</v>
-      </c>
-      <c r="F1" s="22" t="s">
-        <v>473</v>
-      </c>
-      <c r="G1" s="22" t="s">
+      <c r="C2" t="s">
         <v>474</v>
-      </c>
-      <c r="H1" s="22" t="s">
-        <v>478</v>
-      </c>
-      <c r="I1" s="22" t="s">
-        <v>479</v>
-      </c>
-      <c r="J1" s="22" t="s">
-        <v>480</v>
-      </c>
-      <c r="K1" s="22" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>481</v>
-      </c>
-      <c r="B2" t="s">
-        <v>341</v>
-      </c>
-      <c r="C2" t="s">
-        <v>341</v>
       </c>
       <c r="D2" t="s">
         <v>477</v>
       </c>
-      <c r="E2" t="s">
-        <v>341</v>
-      </c>
       <c r="F2" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="G2" t="s">
-        <v>483</v>
-      </c>
-      <c r="H2" t="s">
-        <v>484</v>
-      </c>
-      <c r="I2" t="s">
-        <v>485</v>
-      </c>
-      <c r="J2" t="s">
-        <v>486</v>
-      </c>
-      <c r="K2" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>487</v>
+        <v>407</v>
       </c>
       <c r="B3" t="s">
-        <v>407</v>
+        <v>476</v>
       </c>
       <c r="C3" t="s">
-        <v>407</v>
+        <v>474</v>
       </c>
       <c r="D3" t="s">
         <v>477</v>
       </c>
-      <c r="E3" t="s">
-        <v>407</v>
-      </c>
       <c r="F3" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="G3" t="s">
-        <v>483</v>
-      </c>
-      <c r="H3" t="s">
-        <v>490</v>
-      </c>
-      <c r="I3" t="s">
-        <v>488</v>
-      </c>
-      <c r="J3" t="s">
-        <v>486</v>
-      </c>
-      <c r="K3" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>489</v>
+        <v>427</v>
       </c>
       <c r="B4" t="s">
-        <v>427</v>
+        <v>476</v>
       </c>
       <c r="C4" t="s">
-        <v>427</v>
+        <v>474</v>
       </c>
       <c r="D4" t="s">
         <v>477</v>
       </c>
-      <c r="E4" t="s">
-        <v>427</v>
-      </c>
       <c r="F4" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="G4" t="s">
-        <v>483</v>
-      </c>
-      <c r="H4" t="s">
-        <v>491</v>
-      </c>
-      <c r="I4" t="s">
-        <v>492</v>
-      </c>
-      <c r="J4" t="s">
-        <v>486</v>
-      </c>
-      <c r="K4" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>493</v>
+        <v>433</v>
       </c>
       <c r="B5" t="s">
-        <v>433</v>
+        <v>476</v>
       </c>
       <c r="C5" t="s">
-        <v>433</v>
+        <v>474</v>
       </c>
       <c r="D5" t="s">
         <v>477</v>
       </c>
-      <c r="E5" t="s">
-        <v>433</v>
-      </c>
       <c r="F5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="G5" t="s">
-        <v>483</v>
-      </c>
-      <c r="H5" t="s">
-        <v>494</v>
-      </c>
-      <c r="I5" t="s">
         <v>495</v>
       </c>
-      <c r="J5" t="s">
-        <v>486</v>
-      </c>
-      <c r="K5" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>496</v>
+        <v>401</v>
       </c>
       <c r="B6" t="s">
-        <v>401</v>
+        <v>476</v>
       </c>
       <c r="C6" t="s">
-        <v>401</v>
+        <v>474</v>
       </c>
       <c r="D6" t="s">
         <v>477</v>
       </c>
-      <c r="E6" t="s">
-        <v>401</v>
-      </c>
       <c r="F6" t="s">
         <v>482</v>
       </c>
       <c r="G6" t="s">
-        <v>483</v>
-      </c>
-      <c r="H6" t="s">
-        <v>497</v>
-      </c>
-      <c r="I6" t="s">
-        <v>498</v>
-      </c>
-      <c r="J6" t="s">
-        <v>486</v>
-      </c>
-      <c r="K6" t="s">
-        <v>512</v>
+        <v>496</v>
       </c>
     </row>
   </sheetData>
@@ -3012,10 +2885,10 @@
     </row>
     <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="12" t="s">
-        <v>499</v>
+        <v>483</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>503</v>
+        <v>487</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>31</v>
@@ -3081,10 +2954,10 @@
     </row>
     <row r="9" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="12" t="s">
-        <v>500</v>
+        <v>484</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>504</v>
+        <v>488</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>11</v>
@@ -3096,14 +2969,16 @@
         <v>45</v>
       </c>
       <c r="F9" s="10"/>
-      <c r="G9" s="8"/>
-    </row>
-    <row r="10" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="G9" s="8" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A10" s="12" t="s">
-        <v>501</v>
+        <v>485</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>505</v>
+        <v>489</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>11</v>
@@ -3117,14 +2992,16 @@
       <c r="F10" s="8" t="s">
         <v>290</v>
       </c>
-      <c r="G10" s="8"/>
+      <c r="G10" s="8" t="s">
+        <v>499</v>
+      </c>
     </row>
     <row r="11" spans="1:11" ht="137.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
-        <v>502</v>
+        <v>486</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>506</v>
+        <v>490</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Updates based on CDISC implementation Handbook and test
</commit_message>
<xml_diff>
--- a/Maps/sdtm_mapping_paths.xlsx
+++ b/Maps/sdtm_mapping_paths.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\USDM_SDTM_mapper\Maps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01FF7E84-0502-47C2-8DC0-A24DBAEDA929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06742AC0-AFA4-418B-B776-ADFE4AFB1C75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6225" yWindow="-15525" windowWidth="25590" windowHeight="14265" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="1" r:id="rId1"/>
@@ -1405,9 +1405,6 @@
     <t>study.versions.($EligTxt := function($id) {(eligibilityCriterionItems[id=$id].text)}; studyDesigns.eligibilityCriteria{id: $EligTxt(criterionItemId)})</t>
   </si>
   <si>
-    <t>study.versions.versionIdentifier</t>
-  </si>
-  <si>
     <t>TA</t>
   </si>
   <si>
@@ -1854,15 +1851,6 @@
     <t>study.versions.studyDesigns.objectives[level.code="C85827"].{name: text}</t>
   </si>
   <si>
-    <t>study.versions.studyDesigns.objectives[level.code="C163559"].{name: objectives.endpoint.text}</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.objectives[level.code="C85826"].{name: objectives.endpoint.text}</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.objectives[level.code="C85827"].{name: objectives.endpoint.text}</t>
-  </si>
-  <si>
     <t>study.versions.studyDesigns.indications.{id: label}</t>
   </si>
   <si>
@@ -1973,6 +1961,18 @@
   <si>
     <t>study.versions.studyDesigns.scheduleTimelines.($GetEpochId := function($id) {(instances[id=$id].epochId)}; instances[instanceType="ScheduledDecisionInstance"].
 {epochId: conditionAssignments.condition,"targetEpoch":$GetEpochId(conditionAssignments.conditionTargetId)})</t>
+  </si>
+  <si>
+    <t>$exists(study.versions.versionIdentifier) ? study.versions.versionIdentifier : study.documentedBy[type.code="C70817"].versions.version</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives[level.code="C85826"].{name: endpoints.text}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives[level.code="C85827"].{name: endpoints.text}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives[level.code="C163559"].{name: endpoints.text}</t>
   </si>
 </sst>
 </file>
@@ -2532,7 +2532,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="31" x14ac:dyDescent="0.35">
@@ -2540,23 +2540,23 @@
         <v>324</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="31" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="31" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>422</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>423</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -2586,15 +2586,15 @@
         <v>317</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
+        <v>424</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>425</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>426</v>
       </c>
     </row>
   </sheetData>
@@ -2616,25 +2616,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="22" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="B1" s="22" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>469</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>468</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>493</v>
+      </c>
+      <c r="F1" s="22" t="s">
         <v>471</v>
       </c>
-      <c r="C1" s="22" t="s">
-        <v>473</v>
-      </c>
-      <c r="D1" s="22" t="s">
-        <v>472</v>
-      </c>
-      <c r="E1" s="22" t="s">
-        <v>497</v>
-      </c>
-      <c r="F1" s="22" t="s">
-        <v>475</v>
-      </c>
       <c r="G1" s="22" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -2642,79 +2642,79 @@
         <v>341</v>
       </c>
       <c r="B2" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="C2" t="s">
+        <v>470</v>
+      </c>
+      <c r="D2" t="s">
+        <v>473</v>
+      </c>
+      <c r="F2" t="s">
         <v>474</v>
       </c>
-      <c r="D2" t="s">
-        <v>477</v>
-      </c>
-      <c r="F2" t="s">
-        <v>478</v>
-      </c>
       <c r="G2" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B3" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="C3" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="D3" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="F3" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="G3" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B4" t="s">
+        <v>472</v>
+      </c>
+      <c r="C4" t="s">
+        <v>470</v>
+      </c>
+      <c r="D4" t="s">
+        <v>473</v>
+      </c>
+      <c r="F4" t="s">
         <v>476</v>
       </c>
-      <c r="C4" t="s">
-        <v>474</v>
-      </c>
-      <c r="D4" t="s">
-        <v>477</v>
-      </c>
-      <c r="F4" t="s">
-        <v>480</v>
-      </c>
       <c r="G4" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B5" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="C5" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="D5" t="s">
+        <v>473</v>
+      </c>
+      <c r="F5" t="s">
         <v>477</v>
       </c>
-      <c r="F5" t="s">
-        <v>481</v>
-      </c>
       <c r="G5" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -2722,19 +2722,19 @@
         <v>401</v>
       </c>
       <c r="B6" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="C6" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="D6" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="F6" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="G6" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
     </row>
   </sheetData>
@@ -2805,7 +2805,7 @@
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -2831,7 +2831,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -2857,7 +2857,7 @@
         <v>285</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -2880,15 +2880,15 @@
         <v>286</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="12" t="s">
+        <v>479</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>483</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>487</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>31</v>
@@ -2903,7 +2903,7 @@
         <v>287</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="118" customHeight="1" x14ac:dyDescent="0.35">
@@ -2926,7 +2926,7 @@
         <v>288</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -2949,15 +2949,15 @@
         <v>289</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="12" t="s">
+        <v>480</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>484</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>488</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>11</v>
@@ -2970,15 +2970,15 @@
       </c>
       <c r="F9" s="10"/>
       <c r="G9" s="8" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A10" s="12" t="s">
+        <v>481</v>
+      </c>
+      <c r="B10" s="12" t="s">
         <v>485</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>489</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>11</v>
@@ -2993,15 +2993,15 @@
         <v>290</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="137.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
+        <v>482</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>486</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>490</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>11</v>
@@ -3016,11 +3016,12 @@
         <v>291</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3085,7 +3086,7 @@
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="1"/>
@@ -3111,7 +3112,7 @@
       <c r="F3" s="10"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -3137,7 +3138,7 @@
         <v>311</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3160,7 +3161,7 @@
         <v>312</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3183,7 +3184,7 @@
         <v>292</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3206,7 +3207,7 @@
         <v>293</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3295,7 +3296,7 @@
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="H2" s="8"/>
     </row>
@@ -3318,7 +3319,7 @@
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
       <c r="H3" s="8" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -3341,7 +3342,7 @@
         <v>30</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H4" s="8"/>
     </row>
@@ -3365,7 +3366,7 @@
         <v>33</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="H5" s="8"/>
     </row>
@@ -3389,7 +3390,7 @@
         <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="H6" s="8"/>
     </row>
@@ -3413,7 +3414,7 @@
         <v>285</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="H7" s="8"/>
     </row>
@@ -3437,7 +3438,7 @@
         <v>286</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="H8" s="8"/>
     </row>
@@ -3461,7 +3462,7 @@
         <v>41</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="H9" s="8"/>
     </row>
@@ -3485,7 +3486,7 @@
         <v>43</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="H10" s="8"/>
     </row>
@@ -3573,7 +3574,7 @@
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3709,7 +3710,7 @@
       <c r="F8" s="14"/>
       <c r="G8" s="8"/>
     </row>
-    <row r="9" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>56</v>
       </c>
@@ -3729,11 +3730,12 @@
         <v>57</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>406</v>
+        <v>496</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3806,7 +3808,7 @@
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
@@ -4109,7 +4111,7 @@
         <v>296</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="101.5" x14ac:dyDescent="0.35">
@@ -4128,7 +4130,7 @@
         <v>297</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="H4" s="16" t="s">
         <v>386</v>
@@ -4198,7 +4200,7 @@
       </c>
       <c r="F7" s="17"/>
       <c r="G7" s="5" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4261,7 +4263,7 @@
         <v>340</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4284,7 +4286,7 @@
         <v>300</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4326,7 +4328,7 @@
         <v>301</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4349,7 +4351,7 @@
         <v>122</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="58" x14ac:dyDescent="0.35">
@@ -4372,7 +4374,7 @@
         <v>302</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>349</v>
@@ -4404,7 +4406,7 @@
         <v>303</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>352</v>
@@ -4488,7 +4490,7 @@
         <v>304</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4539,7 +4541,7 @@
         <v>146</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>358</v>
@@ -4567,7 +4569,7 @@
         <v>321</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="H23" t="s">
         <v>347</v>
@@ -4589,7 +4591,7 @@
         <v>305</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
@@ -4608,7 +4610,7 @@
         <v>158</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4666,7 +4668,7 @@
         <v>168</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4689,7 +4691,7 @@
         <v>174</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4712,7 +4714,7 @@
         <v>178</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4838,7 +4840,7 @@
         <v>191</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>461</v>
+        <v>499</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4861,7 +4863,7 @@
         <v>196</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>462</v>
+        <v>497</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4884,7 +4886,7 @@
         <v>199</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>463</v>
+        <v>498</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4967,7 +4969,7 @@
         <v>308</v>
       </c>
       <c r="G41" s="20" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="H41" t="s">
         <v>347</v>
@@ -5051,7 +5053,7 @@
         <v>227</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>380</v>
@@ -5083,7 +5085,7 @@
         <v>230</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
@@ -5102,7 +5104,7 @@
         <v>234</v>
       </c>
       <c r="G47" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5158,7 +5160,7 @@
         <v>310</v>
       </c>
       <c r="G50" s="18" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5233,7 +5235,7 @@
         <v>257</v>
       </c>
       <c r="G53" s="20" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="I53" s="20" t="s">
         <v>374</v>
@@ -5291,16 +5293,16 @@
         <v>264</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="I55" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="J55" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="J55" s="5" t="s">
+      <c r="K55" s="5" t="s">
         <v>413</v>
-      </c>
-      <c r="K55" s="5" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5373,7 +5375,7 @@
         <v>277</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="H58" s="16" t="s">
         <v>348</v>
@@ -5395,16 +5397,16 @@
         <v>281</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I59" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="J59" s="5" t="s">
         <v>415</v>
       </c>
-      <c r="J59" s="5" t="s">
+      <c r="K59" s="5" t="s">
         <v>416</v>
-      </c>
-      <c r="K59" s="5" t="s">
-        <v>417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added ItemDef option to Define
</commit_message>
<xml_diff>
--- a/Maps/sdtm_mapping_paths.xlsx
+++ b/Maps/sdtm_mapping_paths.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\USDM_SDTM_mapper\Maps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F3BB9AB-B628-4DD8-9133-147C9D02B4B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FF2E33-4AE4-4873-9D5B-3D6F42434EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13785" yWindow="-17070" windowWidth="21150" windowHeight="15660" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated mapping and resolveTag capability
</commit_message>
<xml_diff>
--- a/Maps/sdtm_mapping_paths.xlsx
+++ b/Maps/sdtm_mapping_paths.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\USDM_SDTM_mapper\Maps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FF2E33-4AE4-4873-9D5B-3D6F42434EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DECF623C-649C-4F26-9A20-21C6341BB5C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11700" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="502">
   <si>
     <t>Identifier</t>
   </si>
@@ -1270,9 +1270,6 @@
     <t>study.versions.studyInterventions{id: type.codeSystemVersion}</t>
   </si>
   <si>
-    <t>$exists(study.versions.studyDesigns.population.cohorts) ? $count(study.versions.studyDesigns.population.cohorts) : ""</t>
-  </si>
-  <si>
     <t>study.versions.studyDesigns[studyType.code="C16084"].model.code</t>
   </si>
   <si>
@@ -1480,9 +1477,6 @@
     <t>study.versions.studyDesigns.elements.{id: transitionEndRule.text}</t>
   </si>
   <si>
-    <t>$count(study.versions.studyDesigns.arms)</t>
-  </si>
-  <si>
     <t>TV</t>
   </si>
   <si>
@@ -1520,296 +1514,6 @@
   </si>
   <si>
     <t>study.versions.studyDesigns.population.plannedSex.decode</t>
-  </si>
-  <si>
-    <r>
-      <t>$exists</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>study</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>versions</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>studyDesigns</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>characteristics</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>code</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFA00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"C217005"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>])</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> ? "Y" : ""</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>$exists</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>study</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>versions</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>studyDesigns</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>characteristics</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>code</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFA00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"C217004"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>])</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> ? "Y" : ""</t>
-    </r>
   </si>
   <si>
     <t>study.versions.studyInterventions[role.code="C68609"].{name: label}</t>
@@ -1863,12 +1567,6 @@
 $substring($distinct(study.versions.studyDesigns.population.plannedAge.maxValue.unit.standardCode.decode),0,1) &amp;  $substring($distinct(study.versions.studyDesigns.population.cohorts.plannedAge.maxValue.unit.standardCode.decode),0,1)</t>
   </si>
   <si>
-    <t>study.versions.studyInterventions.{name: "P" &amp; minimumResponseDuration.value &amp; $substring(minimumResponseDuration.unit.standardCode.decode,1,1)}</t>
-  </si>
-  <si>
-    <t>$exists(study.versions.studyDesigns.scheduleTimelines[mainTimeline=true].plannedDuration.quantity) ? "P" &amp; study.versions.studyDesigns.scheduleTimelines[mainTimeline=true].plannedDuration.quantity.value &amp; $substring(study.versions.studyDesigns.scheduleTimelines[mainTimeline=true].plannedDuration.quantity.unit.standardCode.decode,1,1)</t>
-  </si>
-  <si>
     <t>study.versions.studyInterventions{name: administrations.duration.quantity.("P"&amp; value &amp; $substring(unit.standardCode.decode,0,1))}</t>
   </si>
   <si>
@@ -1973,6 +1671,31 @@
   </si>
   <si>
     <t>study.versions.studyDesigns.objectives[level.code="C163559"].{name: endpoints.text}</t>
+  </si>
+  <si>
+    <t>study.versions.roles.assignedPersons.{name: personName.text}</t>
+  </si>
+  <si>
+    <t>study.versions.roles@$rl.$rl.assignedPersons.{name: $rl.code.decode}</t>
+  </si>
+  <si>
+    <t>study.versions.studyInterventions.{name: "P" &amp; minimumResponseDuration.value &amp; $substring(minimumResponseDuration.unit.standardCode.decode,0,1)}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.scheduleTimelines[mainTimeline=true].plannedDuration@$pd.
+$pd.$exists(quantity.value) ? "P" &amp; $pd.quantity.value &amp; $substring($pd.quantity.unit.standardCode.decode,0,1)</t>
+  </si>
+  <si>
+    <t>study.versions@$sv.($sv.studyDesigns.$count(arms)&gt;0 ? $sv.studyDesigns.$count(arms))</t>
+  </si>
+  <si>
+    <t>$exists(study.versions.studyDesigns.characteristics[code="C217005"]) ? "Y" : ""</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns@$sd.($sd.population.$count(cohorts)&gt;0 ? $sd.population.$count(cohorts))</t>
+  </si>
+  <si>
+    <t>$exists(study.versions.studyDesigns.characteristics[code="C217004"]) ? "Y" : ""</t>
   </si>
 </sst>
 </file>
@@ -2532,7 +2255,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="31" x14ac:dyDescent="0.35">
@@ -2540,23 +2263,23 @@
         <v>324</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="31" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="31" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>421</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -2586,15 +2309,15 @@
         <v>317</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
+        <v>423</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>424</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -2616,25 +2339,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="22" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="G1" s="22" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -2642,99 +2365,99 @@
         <v>341</v>
       </c>
       <c r="B2" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="C2" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D2" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="F2" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="G2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B3" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="C3" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D3" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="F3" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
       <c r="G3" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B4" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="C4" t="s">
+        <v>464</v>
+      </c>
+      <c r="D4" t="s">
+        <v>467</v>
+      </c>
+      <c r="F4" t="s">
         <v>470</v>
       </c>
-      <c r="D4" t="s">
-        <v>473</v>
-      </c>
-      <c r="F4" t="s">
-        <v>476</v>
-      </c>
       <c r="G4" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B5" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="C5" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D5" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="F5" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="G5" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B6" t="s">
+        <v>466</v>
+      </c>
+      <c r="C6" t="s">
+        <v>464</v>
+      </c>
+      <c r="D6" t="s">
+        <v>467</v>
+      </c>
+      <c r="F6" t="s">
         <v>472</v>
       </c>
-      <c r="C6" t="s">
-        <v>470</v>
-      </c>
-      <c r="D6" t="s">
-        <v>473</v>
-      </c>
-      <c r="F6" t="s">
-        <v>478</v>
-      </c>
       <c r="G6" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
     </row>
   </sheetData>
@@ -2805,7 +2528,7 @@
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -2831,7 +2554,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -2857,7 +2580,7 @@
         <v>285</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -2880,15 +2603,15 @@
         <v>286</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="12" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>31</v>
@@ -2903,7 +2626,7 @@
         <v>287</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="118" customHeight="1" x14ac:dyDescent="0.35">
@@ -2926,7 +2649,7 @@
         <v>288</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -2949,15 +2672,15 @@
         <v>289</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="12" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>11</v>
@@ -2970,15 +2693,15 @@
       </c>
       <c r="F9" s="10"/>
       <c r="G9" s="8" t="s">
-        <v>494</v>
+        <v>488</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A10" s="12" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>11</v>
@@ -2993,15 +2716,15 @@
         <v>290</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="137.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>11</v>
@@ -3016,7 +2739,7 @@
         <v>291</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
   </sheetData>
@@ -3086,7 +2809,7 @@
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="1"/>
@@ -3112,7 +2835,7 @@
       <c r="F3" s="10"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -3138,7 +2861,7 @@
         <v>311</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3161,7 +2884,7 @@
         <v>312</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3184,7 +2907,7 @@
         <v>292</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3207,7 +2930,7 @@
         <v>293</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -3296,7 +3019,7 @@
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="H2" s="8"/>
     </row>
@@ -3319,7 +3042,7 @@
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
       <c r="H3" s="8" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -3342,7 +3065,7 @@
         <v>30</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="H4" s="8"/>
     </row>
@@ -3366,7 +3089,7 @@
         <v>33</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="H5" s="8"/>
     </row>
@@ -3390,7 +3113,7 @@
         <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="H6" s="8"/>
     </row>
@@ -3414,7 +3137,7 @@
         <v>285</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="H7" s="8"/>
     </row>
@@ -3438,7 +3161,7 @@
         <v>286</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="H8" s="8"/>
     </row>
@@ -3462,7 +3185,7 @@
         <v>41</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="H9" s="8"/>
     </row>
@@ -3486,7 +3209,7 @@
         <v>43</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="H10" s="8"/>
     </row>
@@ -3574,7 +3297,7 @@
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3596,7 +3319,7 @@
       <c r="F3" s="14"/>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3619,7 +3342,7 @@
         <v>47</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -3642,7 +3365,7 @@
         <v>49</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3665,7 +3388,7 @@
         <v>51</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3688,7 +3411,7 @@
         <v>53</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -3730,7 +3453,7 @@
         <v>57</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
     </row>
   </sheetData>
@@ -3808,7 +3531,7 @@
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
@@ -4111,7 +3834,7 @@
         <v>296</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="101.5" x14ac:dyDescent="0.35">
@@ -4130,10 +3853,10 @@
         <v>297</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="58" x14ac:dyDescent="0.35">
@@ -4200,7 +3923,7 @@
       </c>
       <c r="F7" s="17"/>
       <c r="G7" s="5" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4222,6 +3945,9 @@
       <c r="F8" s="17" t="s">
         <v>100</v>
       </c>
+      <c r="G8" s="5" t="s">
+        <v>494</v>
+      </c>
     </row>
     <row r="9" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="16" t="s">
@@ -4242,6 +3968,9 @@
       <c r="F9" s="17" t="s">
         <v>104</v>
       </c>
+      <c r="G9" s="5" t="s">
+        <v>495</v>
+      </c>
     </row>
     <row r="10" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
@@ -4263,7 +3992,7 @@
         <v>340</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>463</v>
+        <v>496</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4286,7 +4015,7 @@
         <v>300</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4305,7 +4034,7 @@
         <v>116</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4328,7 +4057,7 @@
         <v>301</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
@@ -4351,7 +4080,7 @@
         <v>122</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="58" x14ac:dyDescent="0.35">
@@ -4374,7 +4103,7 @@
         <v>302</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>349</v>
@@ -4406,7 +4135,7 @@
         <v>303</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>352</v>
@@ -4434,7 +4163,7 @@
         <v>131</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4468,10 +4197,10 @@
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="17" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="58" x14ac:dyDescent="0.35">
@@ -4490,7 +4219,7 @@
         <v>304</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4541,7 +4270,7 @@
         <v>146</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>358</v>
@@ -4553,7 +4282,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="87" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A23" s="16" t="s">
         <v>149</v>
       </c>
@@ -4569,7 +4298,7 @@
         <v>321</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>464</v>
+        <v>497</v>
       </c>
       <c r="H23" t="s">
         <v>347</v>
@@ -4590,11 +4319,11 @@
       <c r="F24" s="17" t="s">
         <v>305</v>
       </c>
-      <c r="G24" s="18" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G24" s="20" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="16" t="s">
         <v>155</v>
       </c>
@@ -4610,7 +4339,7 @@
         <v>158</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>431</v>
+        <v>498</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4629,7 +4358,7 @@
         <v>159</v>
       </c>
       <c r="G26" s="20" t="s">
-        <v>361</v>
+        <v>500</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4668,7 +4397,7 @@
         <v>168</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4691,7 +4420,7 @@
         <v>174</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4714,7 +4443,7 @@
         <v>178</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4736,13 +4465,13 @@
         <v>333</v>
       </c>
       <c r="I31" t="s">
+        <v>361</v>
+      </c>
+      <c r="J31" t="s">
         <v>362</v>
       </c>
-      <c r="J31" t="s">
+      <c r="K31" t="s">
         <v>363</v>
-      </c>
-      <c r="K31" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4764,13 +4493,13 @@
         <v>334</v>
       </c>
       <c r="I32" s="20" t="s">
+        <v>364</v>
+      </c>
+      <c r="J32" s="20" t="s">
         <v>365</v>
       </c>
-      <c r="J32" s="20" t="s">
+      <c r="K32" s="20" t="s">
         <v>366</v>
-      </c>
-      <c r="K32" s="20" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4811,13 +4540,13 @@
         <v>336</v>
       </c>
       <c r="I34" s="20" t="s">
+        <v>367</v>
+      </c>
+      <c r="J34" s="20" t="s">
         <v>368</v>
       </c>
-      <c r="J34" s="20" t="s">
+      <c r="K34" s="20" t="s">
         <v>369</v>
-      </c>
-      <c r="K34" s="20" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4840,7 +4569,7 @@
         <v>191</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4863,7 +4592,7 @@
         <v>196</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4886,7 +4615,7 @@
         <v>199</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4907,7 +4636,7 @@
         <v>202</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -4926,7 +4655,7 @@
         <v>205</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -4969,7 +4698,7 @@
         <v>308</v>
       </c>
       <c r="G41" s="20" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="H41" t="s">
         <v>347</v>
@@ -4991,7 +4720,7 @@
         <v>217</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
@@ -5010,7 +4739,7 @@
         <v>221</v>
       </c>
       <c r="G43" s="20" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -5053,16 +4782,16 @@
         <v>227</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="I45" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="J45" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="J45" s="5" t="s">
+      <c r="K45" s="5" t="s">
         <v>381</v>
-      </c>
-      <c r="K45" s="5" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="58" x14ac:dyDescent="0.35">
@@ -5085,7 +4814,7 @@
         <v>230</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
@@ -5104,7 +4833,7 @@
         <v>234</v>
       </c>
       <c r="G47" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5123,7 +4852,7 @@
         <v>309</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5160,7 +4889,7 @@
         <v>310</v>
       </c>
       <c r="G50" s="18" t="s">
-        <v>446</v>
+        <v>501</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5179,16 +4908,16 @@
         <v>249</v>
       </c>
       <c r="G51" t="s">
+        <v>392</v>
+      </c>
+      <c r="I51" t="s">
         <v>393</v>
       </c>
-      <c r="I51" t="s">
+      <c r="J51" t="s">
         <v>394</v>
       </c>
-      <c r="J51" t="s">
+      <c r="K51" t="s">
         <v>395</v>
-      </c>
-      <c r="K51" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
@@ -5210,13 +4939,13 @@
         <v>331</v>
       </c>
       <c r="I52" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="J52" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="J52" s="5" t="s">
+      <c r="K52" s="5" t="s">
         <v>372</v>
-      </c>
-      <c r="K52" s="5" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
@@ -5235,16 +4964,16 @@
         <v>257</v>
       </c>
       <c r="G53" s="20" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="I53" s="20" t="s">
+        <v>373</v>
+      </c>
+      <c r="J53" s="20" t="s">
         <v>374</v>
       </c>
-      <c r="J53" s="20" t="s">
+      <c r="K53" s="20" t="s">
         <v>375</v>
-      </c>
-      <c r="K53" s="20" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5263,16 +4992,16 @@
         <v>258</v>
       </c>
       <c r="G54" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="I54" s="5" t="s">
         <v>397</v>
       </c>
-      <c r="I54" s="5" t="s">
+      <c r="J54" s="5" t="s">
         <v>398</v>
       </c>
-      <c r="J54" s="5" t="s">
+      <c r="K54" s="5" t="s">
         <v>399</v>
-      </c>
-      <c r="K54" s="5" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -5293,16 +5022,16 @@
         <v>264</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="I55" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="J55" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="J55" s="5" t="s">
+      <c r="K55" s="5" t="s">
         <v>412</v>
-      </c>
-      <c r="K55" s="5" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -5346,13 +5075,13 @@
         <v>347</v>
       </c>
       <c r="I57" t="s">
+        <v>376</v>
+      </c>
+      <c r="J57" t="s">
         <v>377</v>
       </c>
-      <c r="J57" t="s">
+      <c r="K57" t="s">
         <v>378</v>
-      </c>
-      <c r="K57" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -5375,7 +5104,7 @@
         <v>277</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="H58" s="16" t="s">
         <v>348</v>
@@ -5397,16 +5126,16 @@
         <v>281</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="I59" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="J59" s="5" t="s">
         <v>414</v>
       </c>
-      <c r="J59" s="5" t="s">
+      <c r="K59" s="5" t="s">
         <v>415</v>
-      </c>
-      <c r="K59" s="5" t="s">
-        <v>416</v>
       </c>
     </row>
   </sheetData>

</xml_diff>